<commit_message>
Add VSCode launch config and update spreadsheets
Add a .vscode/launch.json template (empty configurations) and update two binary Excel files: Planilla_SprintBacklog_YZ.xlsx and Project-roadmap_YZ.xlsx. These changes introduce an editor debug config file and update project backlog/roadmap documents; no source code was modified.
</commit_message>
<xml_diff>
--- a/Planilla_SprintBacklog_YZ.xlsx
+++ b/Planilla_SprintBacklog_YZ.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yolze\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9A69C915-3460-40B5-9444-16239C28E8C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE2B488E-205F-4322-ACEC-C840FF8483F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-105" yWindow="0" windowWidth="19410" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -220,36 +220,18 @@
     <t>Baja</t>
   </si>
   <si>
-    <t>Calendario UI</t>
-  </si>
-  <si>
-    <t>Galería Multimedia</t>
-  </si>
-  <si>
     <t>Detalle Habitación</t>
   </si>
   <si>
     <t>Módulo Login</t>
   </si>
   <si>
-    <t>Lógica Precios</t>
-  </si>
-  <si>
-    <t>API de Pago</t>
-  </si>
-  <si>
     <t>Selector I18n</t>
   </si>
   <si>
     <t>Layout CSS</t>
   </si>
   <si>
-    <t>Panel de Tarifas</t>
-  </si>
-  <si>
-    <t>Generador QR</t>
-  </si>
-  <si>
     <t>Servicio SMTP</t>
   </si>
   <si>
@@ -263,6 +245,24 @@
   </si>
   <si>
     <t>Módulo RBAC</t>
+  </si>
+  <si>
+    <t>Mockup Figma (Landing) + Diagrama de Actividades UML</t>
+  </si>
+  <si>
+    <t>Mockup Figma (Catálogo Grid)</t>
+  </si>
+  <si>
+    <t>Diagrama de Estados UML (Habitación)</t>
+  </si>
+  <si>
+    <t>Mockup Figma (Checkout) + Diagrama de Secuencia UML</t>
+  </si>
+  <si>
+    <t>Mockup Figma (Dashboard Admin)</t>
+  </si>
+  <si>
+    <t>Diagrama de Secuencia UML (QR)</t>
   </si>
 </sst>
 </file>
@@ -420,12 +420,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -441,7 +435,13 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -890,54 +890,54 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="12"/>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
-      <c r="F1" s="11" t="s">
+      <c r="B1" s="18"/>
+      <c r="C1" s="18"/>
+      <c r="D1" s="18"/>
+      <c r="E1" s="18"/>
+      <c r="F1" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="G1" s="11"/>
-      <c r="H1" s="11"/>
-      <c r="I1" s="11"/>
-      <c r="J1" s="11"/>
-      <c r="K1" s="11"/>
+      <c r="G1" s="17"/>
+      <c r="H1" s="17"/>
+      <c r="I1" s="17"/>
+      <c r="J1" s="17"/>
+      <c r="K1" s="17"/>
     </row>
     <row r="2" spans="1:11" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="13" t="s">
+      <c r="A2" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="13" t="s">
+      <c r="B2" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="13" t="s">
+      <c r="C2" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="D2" s="14" t="s">
+      <c r="D2" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="E2" s="13" t="s">
+      <c r="E2" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="F2" s="15" t="s">
+      <c r="F2" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="G2" s="15" t="s">
+      <c r="G2" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="H2" s="15" t="s">
+      <c r="H2" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="I2" s="13" t="s">
+      <c r="I2" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="J2" s="13" t="s">
+      <c r="J2" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="K2" s="13" t="s">
+      <c r="K2" s="11" t="s">
         <v>12</v>
       </c>
     </row>
@@ -945,34 +945,34 @@
       <c r="A3" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="B3" s="16" t="s">
+      <c r="B3" s="14" t="s">
         <v>33</v>
       </c>
-      <c r="C3" s="16" t="s">
+      <c r="C3" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="D3" s="16" t="s">
-        <v>60</v>
-      </c>
-      <c r="E3" s="16" t="s">
+      <c r="D3" s="14" t="s">
+        <v>69</v>
+      </c>
+      <c r="E3" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="F3" s="17">
+      <c r="F3" s="15">
         <v>8</v>
       </c>
-      <c r="G3" s="17" t="s">
+      <c r="G3" s="15" t="s">
         <v>57</v>
       </c>
-      <c r="H3" s="18">
+      <c r="H3" s="16">
         <v>1</v>
       </c>
-      <c r="I3" s="17">
+      <c r="I3" s="15">
         <v>1</v>
       </c>
-      <c r="J3" s="16" t="s">
+      <c r="J3" s="14" t="s">
         <v>31</v>
       </c>
-      <c r="K3" s="16" t="s">
+      <c r="K3" s="14" t="s">
         <v>14</v>
       </c>
     </row>
@@ -980,34 +980,34 @@
       <c r="A4" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="B4" s="16" t="s">
+      <c r="B4" s="14" t="s">
         <v>34</v>
       </c>
-      <c r="C4" s="16" t="s">
+      <c r="C4" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="D4" s="16" t="s">
-        <v>61</v>
-      </c>
-      <c r="E4" s="16" t="s">
+      <c r="D4" s="14" t="s">
+        <v>70</v>
+      </c>
+      <c r="E4" s="14" t="s">
         <v>52</v>
       </c>
-      <c r="F4" s="17">
+      <c r="F4" s="15">
         <v>5</v>
       </c>
-      <c r="G4" s="17" t="s">
+      <c r="G4" s="15" t="s">
         <v>56</v>
       </c>
-      <c r="H4" s="18">
+      <c r="H4" s="16">
         <v>1</v>
       </c>
-      <c r="I4" s="17">
+      <c r="I4" s="15">
         <v>1</v>
       </c>
-      <c r="J4" s="16" t="s">
+      <c r="J4" s="14" t="s">
         <v>31</v>
       </c>
-      <c r="K4" s="16" t="s">
+      <c r="K4" s="14" t="s">
         <v>14</v>
       </c>
     </row>
@@ -1015,34 +1015,34 @@
       <c r="A5" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="B5" s="16" t="s">
+      <c r="B5" s="14" t="s">
         <v>35</v>
       </c>
-      <c r="C5" s="16" t="s">
+      <c r="C5" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="D5" s="16" t="s">
-        <v>62</v>
-      </c>
-      <c r="E5" s="16" t="s">
+      <c r="D5" s="14" t="s">
+        <v>60</v>
+      </c>
+      <c r="E5" s="14" t="s">
         <v>52</v>
       </c>
-      <c r="F5" s="17">
+      <c r="F5" s="15">
         <v>5</v>
       </c>
-      <c r="G5" s="17" t="s">
+      <c r="G5" s="15" t="s">
         <v>58</v>
       </c>
-      <c r="H5" s="18">
+      <c r="H5" s="16">
         <v>1</v>
       </c>
-      <c r="I5" s="17">
+      <c r="I5" s="15">
         <v>1</v>
       </c>
-      <c r="J5" s="16" t="s">
+      <c r="J5" s="14" t="s">
         <v>31</v>
       </c>
-      <c r="K5" s="16" t="s">
+      <c r="K5" s="14" t="s">
         <v>14</v>
       </c>
     </row>
@@ -1050,34 +1050,34 @@
       <c r="A6" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="B6" s="16" t="s">
+      <c r="B6" s="14" t="s">
         <v>36</v>
       </c>
-      <c r="C6" s="16" t="s">
+      <c r="C6" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="D6" s="16" t="s">
-        <v>63</v>
-      </c>
-      <c r="E6" s="16" t="s">
+      <c r="D6" s="14" t="s">
+        <v>61</v>
+      </c>
+      <c r="E6" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="F6" s="17">
+      <c r="F6" s="15">
         <v>8</v>
       </c>
-      <c r="G6" s="17" t="s">
+      <c r="G6" s="15" t="s">
         <v>55</v>
       </c>
-      <c r="H6" s="18">
+      <c r="H6" s="16">
         <v>1</v>
       </c>
-      <c r="I6" s="17">
+      <c r="I6" s="15">
         <v>1</v>
       </c>
-      <c r="J6" s="16" t="s">
+      <c r="J6" s="14" t="s">
         <v>31</v>
       </c>
-      <c r="K6" s="16" t="s">
+      <c r="K6" s="14" t="s">
         <v>14</v>
       </c>
     </row>
@@ -1085,34 +1085,34 @@
       <c r="A7" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="B7" s="16" t="s">
+      <c r="B7" s="14" t="s">
         <v>37</v>
       </c>
-      <c r="C7" s="16" t="s">
+      <c r="C7" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="D7" s="16" t="s">
-        <v>64</v>
-      </c>
-      <c r="E7" s="16" t="s">
+      <c r="D7" s="14" t="s">
+        <v>71</v>
+      </c>
+      <c r="E7" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="F7" s="17">
+      <c r="F7" s="15">
         <v>5</v>
       </c>
-      <c r="G7" s="17" t="s">
+      <c r="G7" s="15" t="s">
         <v>56</v>
       </c>
-      <c r="H7" s="18">
+      <c r="H7" s="16">
         <v>1</v>
       </c>
-      <c r="I7" s="17">
+      <c r="I7" s="15">
         <v>1</v>
       </c>
-      <c r="J7" s="16" t="s">
+      <c r="J7" s="14" t="s">
         <v>31</v>
       </c>
-      <c r="K7" s="16" t="s">
+      <c r="K7" s="14" t="s">
         <v>14</v>
       </c>
     </row>
@@ -1120,34 +1120,34 @@
       <c r="A8" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="B8" s="16" t="s">
+      <c r="B8" s="14" t="s">
         <v>38</v>
       </c>
-      <c r="C8" s="16" t="s">
+      <c r="C8" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="D8" s="16" t="s">
-        <v>65</v>
-      </c>
-      <c r="E8" s="16" t="s">
+      <c r="D8" s="14" t="s">
+        <v>72</v>
+      </c>
+      <c r="E8" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="F8" s="17">
+      <c r="F8" s="15">
         <v>13</v>
       </c>
-      <c r="G8" s="17" t="s">
+      <c r="G8" s="15" t="s">
         <v>54</v>
       </c>
-      <c r="H8" s="18">
+      <c r="H8" s="16">
         <v>1</v>
       </c>
-      <c r="I8" s="17">
+      <c r="I8" s="15">
         <v>2</v>
       </c>
-      <c r="J8" s="16" t="s">
+      <c r="J8" s="14" t="s">
         <v>31</v>
       </c>
-      <c r="K8" s="16" t="s">
+      <c r="K8" s="14" t="s">
         <v>14</v>
       </c>
     </row>
@@ -1155,34 +1155,34 @@
       <c r="A9" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="B9" s="16" t="s">
+      <c r="B9" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="C9" s="16" t="s">
+      <c r="C9" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="D9" s="16" t="s">
-        <v>66</v>
-      </c>
-      <c r="E9" s="16" t="s">
+      <c r="D9" s="14" t="s">
+        <v>62</v>
+      </c>
+      <c r="E9" s="14" t="s">
         <v>52</v>
       </c>
-      <c r="F9" s="17">
+      <c r="F9" s="15">
         <v>3</v>
       </c>
-      <c r="G9" s="17" t="s">
+      <c r="G9" s="15" t="s">
         <v>58</v>
       </c>
-      <c r="H9" s="18">
+      <c r="H9" s="16">
         <v>1</v>
       </c>
-      <c r="I9" s="17">
+      <c r="I9" s="15">
         <v>2</v>
       </c>
-      <c r="J9" s="16" t="s">
+      <c r="J9" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="K9" s="16" t="s">
+      <c r="K9" s="14" t="s">
         <v>14</v>
       </c>
     </row>
@@ -1190,34 +1190,34 @@
       <c r="A10" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="B10" s="16" t="s">
+      <c r="B10" s="14" t="s">
         <v>40</v>
       </c>
-      <c r="C10" s="16" t="s">
+      <c r="C10" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="D10" s="16" t="s">
-        <v>67</v>
-      </c>
-      <c r="E10" s="16" t="s">
+      <c r="D10" s="14" t="s">
+        <v>63</v>
+      </c>
+      <c r="E10" s="14" t="s">
         <v>52</v>
       </c>
-      <c r="F10" s="17">
+      <c r="F10" s="15">
         <v>8</v>
       </c>
-      <c r="G10" s="17" t="s">
+      <c r="G10" s="15" t="s">
         <v>55</v>
       </c>
-      <c r="H10" s="18">
+      <c r="H10" s="16">
         <v>1</v>
       </c>
-      <c r="I10" s="17">
+      <c r="I10" s="15">
         <v>2</v>
       </c>
-      <c r="J10" s="16" t="s">
+      <c r="J10" s="14" t="s">
         <v>31</v>
       </c>
-      <c r="K10" s="16" t="s">
+      <c r="K10" s="14" t="s">
         <v>14</v>
       </c>
     </row>
@@ -1225,34 +1225,34 @@
       <c r="A11" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="B11" s="16" t="s">
+      <c r="B11" s="14" t="s">
         <v>41</v>
       </c>
-      <c r="C11" s="16" t="s">
+      <c r="C11" s="14" t="s">
         <v>49</v>
       </c>
-      <c r="D11" s="16" t="s">
-        <v>68</v>
-      </c>
-      <c r="E11" s="16" t="s">
+      <c r="D11" s="14" t="s">
+        <v>73</v>
+      </c>
+      <c r="E11" s="14" t="s">
         <v>53</v>
       </c>
-      <c r="F11" s="17">
+      <c r="F11" s="15">
         <v>5</v>
       </c>
-      <c r="G11" s="17" t="s">
+      <c r="G11" s="15" t="s">
         <v>56</v>
       </c>
-      <c r="H11" s="18">
+      <c r="H11" s="16">
         <v>1</v>
       </c>
-      <c r="I11" s="17">
+      <c r="I11" s="15">
         <v>2</v>
       </c>
-      <c r="J11" s="16" t="s">
+      <c r="J11" s="14" t="s">
         <v>31</v>
       </c>
-      <c r="K11" s="16" t="s">
+      <c r="K11" s="14" t="s">
         <v>14</v>
       </c>
     </row>
@@ -1260,34 +1260,34 @@
       <c r="A12" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="B12" s="16" t="s">
+      <c r="B12" s="14" t="s">
         <v>42</v>
       </c>
-      <c r="C12" s="16" t="s">
+      <c r="C12" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="D12" s="16" t="s">
-        <v>69</v>
-      </c>
-      <c r="E12" s="16" t="s">
+      <c r="D12" s="14" t="s">
+        <v>74</v>
+      </c>
+      <c r="E12" s="14" t="s">
         <v>52</v>
       </c>
-      <c r="F12" s="17">
+      <c r="F12" s="15">
         <v>13</v>
       </c>
-      <c r="G12" s="17" t="s">
+      <c r="G12" s="15" t="s">
         <v>57</v>
       </c>
-      <c r="H12" s="18">
+      <c r="H12" s="16">
         <v>1</v>
       </c>
-      <c r="I12" s="17">
+      <c r="I12" s="15">
         <v>3</v>
       </c>
-      <c r="J12" s="16" t="s">
+      <c r="J12" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="K12" s="16" t="s">
+      <c r="K12" s="14" t="s">
         <v>14</v>
       </c>
     </row>
@@ -1295,34 +1295,34 @@
       <c r="A13" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="B13" s="16" t="s">
+      <c r="B13" s="14" t="s">
         <v>43</v>
       </c>
-      <c r="C13" s="16" t="s">
+      <c r="C13" s="14" t="s">
         <v>50</v>
       </c>
-      <c r="D13" s="16" t="s">
-        <v>70</v>
-      </c>
-      <c r="E13" s="16" t="s">
+      <c r="D13" s="14" t="s">
+        <v>64</v>
+      </c>
+      <c r="E13" s="14" t="s">
         <v>52</v>
       </c>
-      <c r="F13" s="17">
+      <c r="F13" s="15">
         <v>5</v>
       </c>
-      <c r="G13" s="17" t="s">
+      <c r="G13" s="15" t="s">
         <v>58</v>
       </c>
-      <c r="H13" s="18">
+      <c r="H13" s="16">
         <v>1</v>
       </c>
-      <c r="I13" s="17">
+      <c r="I13" s="15">
         <v>3</v>
       </c>
-      <c r="J13" s="16" t="s">
+      <c r="J13" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="K13" s="16" t="s">
+      <c r="K13" s="14" t="s">
         <v>14</v>
       </c>
     </row>
@@ -1330,34 +1330,34 @@
       <c r="A14" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="B14" s="16" t="s">
+      <c r="B14" s="14" t="s">
         <v>44</v>
       </c>
-      <c r="C14" s="16" t="s">
+      <c r="C14" s="14" t="s">
         <v>49</v>
       </c>
-      <c r="D14" s="16" t="s">
-        <v>71</v>
-      </c>
-      <c r="E14" s="16" t="s">
+      <c r="D14" s="14" t="s">
+        <v>65</v>
+      </c>
+      <c r="E14" s="14" t="s">
         <v>53</v>
       </c>
-      <c r="F14" s="17">
+      <c r="F14" s="15">
         <v>8</v>
       </c>
-      <c r="G14" s="17" t="s">
+      <c r="G14" s="15" t="s">
         <v>55</v>
       </c>
-      <c r="H14" s="18">
+      <c r="H14" s="16">
         <v>1</v>
       </c>
-      <c r="I14" s="17">
+      <c r="I14" s="15">
         <v>3</v>
       </c>
-      <c r="J14" s="16" t="s">
+      <c r="J14" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="K14" s="16" t="s">
+      <c r="K14" s="14" t="s">
         <v>14</v>
       </c>
     </row>
@@ -1365,34 +1365,34 @@
       <c r="A15" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="B15" s="16" t="s">
+      <c r="B15" s="14" t="s">
         <v>45</v>
       </c>
-      <c r="C15" s="16" t="s">
+      <c r="C15" s="14" t="s">
         <v>49</v>
       </c>
-      <c r="D15" s="16" t="s">
-        <v>72</v>
-      </c>
-      <c r="E15" s="16" t="s">
+      <c r="D15" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="E15" s="14" t="s">
         <v>53</v>
       </c>
-      <c r="F15" s="17">
+      <c r="F15" s="15">
         <v>5</v>
       </c>
-      <c r="G15" s="17" t="s">
+      <c r="G15" s="15" t="s">
         <v>56</v>
       </c>
-      <c r="H15" s="18">
+      <c r="H15" s="16">
         <v>1</v>
       </c>
-      <c r="I15" s="17">
+      <c r="I15" s="15">
         <v>3</v>
       </c>
-      <c r="J15" s="16" t="s">
+      <c r="J15" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="K15" s="16" t="s">
+      <c r="K15" s="14" t="s">
         <v>14</v>
       </c>
     </row>
@@ -1400,34 +1400,34 @@
       <c r="A16" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="B16" s="16" t="s">
+      <c r="B16" s="14" t="s">
         <v>46</v>
       </c>
-      <c r="C16" s="16" t="s">
+      <c r="C16" s="14" t="s">
         <v>49</v>
       </c>
-      <c r="D16" s="16" t="s">
-        <v>73</v>
-      </c>
-      <c r="E16" s="16" t="s">
+      <c r="D16" s="14" t="s">
+        <v>67</v>
+      </c>
+      <c r="E16" s="14" t="s">
         <v>53</v>
       </c>
-      <c r="F16" s="17">
+      <c r="F16" s="15">
         <v>5</v>
       </c>
-      <c r="G16" s="17" t="s">
+      <c r="G16" s="15" t="s">
         <v>58</v>
       </c>
-      <c r="H16" s="18">
+      <c r="H16" s="16">
         <v>1</v>
       </c>
-      <c r="I16" s="17">
+      <c r="I16" s="15">
         <v>3</v>
       </c>
-      <c r="J16" s="16" t="s">
+      <c r="J16" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="K16" s="16" t="s">
+      <c r="K16" s="14" t="s">
         <v>14</v>
       </c>
     </row>
@@ -1435,34 +1435,34 @@
       <c r="A17" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="B17" s="16" t="s">
+      <c r="B17" s="14" t="s">
         <v>47</v>
       </c>
-      <c r="C17" s="16" t="s">
+      <c r="C17" s="14" t="s">
         <v>49</v>
       </c>
-      <c r="D17" s="16" t="s">
-        <v>74</v>
-      </c>
-      <c r="E17" s="16" t="s">
+      <c r="D17" s="14" t="s">
+        <v>68</v>
+      </c>
+      <c r="E17" s="14" t="s">
         <v>53</v>
       </c>
-      <c r="F17" s="17">
+      <c r="F17" s="15">
         <v>3</v>
       </c>
-      <c r="G17" s="17" t="s">
+      <c r="G17" s="15" t="s">
         <v>58</v>
       </c>
-      <c r="H17" s="18">
+      <c r="H17" s="16">
         <v>1</v>
       </c>
-      <c r="I17" s="17">
+      <c r="I17" s="15">
         <v>3</v>
       </c>
-      <c r="J17" s="16" t="s">
+      <c r="J17" s="14" t="s">
         <v>59</v>
       </c>
-      <c r="K17" s="16" t="s">
+      <c r="K17" s="14" t="s">
         <v>14</v>
       </c>
     </row>

</xml_diff>